<commit_message>
fix: verification appendix summary showed stale 1,004 fleet
Final audit caught the appendix Summary still reading 'Total buses 1044 ->
1004' while every other RTO surface shows 1,011. Patched to 'Total buses
(v3.4.4 distances -> v3.4.5 measured cycles) 1044 -> 1011' — honest full
chain, no standalone stale number.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/route-rationalization-kashmir/Kashmir_Route_Verification_Appendix_v3.4.5_RTO.xlsx
+++ b/public/route-rationalization-kashmir/Kashmir_Route_Verification_Appendix_v3.4.5_RTO.xlsx
@@ -518,6 +518,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr"/>
       <c r="B4" s="3" t="inlineStr"/>
@@ -694,14 +695,14 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Total buses</t>
+          <t>Total buses (v3.4.4 distances → v3.4.5 measured cycles)</t>
         </is>
       </c>
       <c r="B17" s="3" t="n">
         <v>1044</v>
       </c>
       <c r="C17" s="3" t="n">
-        <v>1004</v>
+        <v>1011</v>
       </c>
     </row>
     <row r="18">

</xml_diff>